<commit_message>
irrelevante kapitel entfernt, IDE und Arduino Vorgänger hinzugefügt
hab paar irrelevante kapitel entfernt und die arduino und IDE Beschreibung von unseren vorgängern hinzugefügt. muss aber noch acronyme einbinden die fehlen, deswegen fehlermeldung beim kompilieren
</commit_message>
<xml_diff>
--- a/LaTeXTemplate/author.xlsx
+++ b/LaTeXTemplate/author.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Wings-Hub\ML24\ML24-EX01-KeywordSpotting\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hanna\Documents\GitHub\Handbuch\LaTeXTemplate\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B97044E-310F-4B56-BC6B-D0357C72CC2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="45" windowWidth="15960" windowHeight="18075"/>
+    <workbookView xWindow="3075" yWindow="3075" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Export Summary" sheetId="1" r:id="rId1"/>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="76">
   <si>
     <t>This document was exported from Numbers. Each table was converted to an Excel worksheet. All other objects on each Numbers sheet were placed on separate worksheets. Please be aware that formula calculations may differ in Excel.</t>
   </si>
@@ -43,19 +44,9 @@
     <t>Table 1</t>
   </si>
   <si>
-    <t>Keyword Spotting with Arduino Nano 33 BLE Sense</t>
-  </si>
-  <si>
     <t>Short Description</t>
   </si>
   <si>
-    <t>In this project, you’ll train a machine learning model to recognize certain keywords
-(e.g., Yes, No). The model is loaded onto your Nano 33 BLE
-board, which has built-in Bluetooth and a microphone—perfect for capturing audio
-input. When the board detects a keyword, it triggers an action, such as blinking an
-LED</t>
-  </si>
-  <si>
     <t>github Project</t>
   </si>
   <si>
@@ -86,9 +77,6 @@
     <t>Study Course:</t>
   </si>
   <si>
-    <t>Business Intelligen ans Data Analytics</t>
-  </si>
-  <si>
     <t>Semester:</t>
   </si>
   <si>
@@ -146,19 +134,10 @@
     <t xml:space="preserve">Home: </t>
   </si>
   <si>
-    <t>&lt;04921 123 456&gt;</t>
-  </si>
-  <si>
     <t xml:space="preserve">Study: </t>
   </si>
   <si>
-    <t>&lt;04921 807 1429&gt;</t>
-  </si>
-  <si>
     <t xml:space="preserve">Workplace: </t>
-  </si>
-  <si>
-    <t>&lt;04921 807 1428&gt;</t>
   </si>
   <si>
     <t>Supervisor workplace:</t>
@@ -190,15 +169,6 @@
     <t>Second examiner:</t>
   </si>
   <si>
-    <t>&lt;Prof. Dr. Carla Columna&gt;</t>
-  </si>
-  <si>
-    <t>&lt;00494921 807-1001&gt;</t>
-  </si>
-  <si>
-    <t>&lt;albert.einstein@hs-emden-leer.de&gt;</t>
-  </si>
-  <si>
     <t>Outstanding examinations:</t>
   </si>
   <si>
@@ -208,44 +178,106 @@
     <t>Student 2</t>
   </si>
   <si>
-    <t>ML &amp; Project T</t>
-  </si>
-  <si>
-    <t>&lt;Hochschule Emden/Leer&gt; or &lt; VW Wolfsburg&gt; or &lt;...&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Fachbereich Technik&gt;  or &lt;Strak&gt; or &lt;...&gt;</t>
-  </si>
-  <si>
     <t>Student 3</t>
   </si>
   <si>
-    <t>Wings</t>
-  </si>
-  <si>
-    <t>Elmar</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> &lt;5&gt; or &lt;10&gt;</t>
-  </si>
-  <si>
     <t>&lt;01.01.2000&gt;</t>
   </si>
   <si>
-    <t>&lt;Steinweg 15&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Einstein, Albert&gt;</t>
-  </si>
-  <si>
-    <t>ML24-04 Keyword Spotting with an Arduino Nano 33 BLE Sense</t>
+    <t>Ansteuerung eines Schrittmotors mit einem Arduino Nano 33 BLE Sense</t>
+  </si>
+  <si>
+    <t>In diesem Projekt wurde mittels eines Arduino Nano 33 BLE Sense die Ansteuerung eines Schrittmotors an einem CNC-Tisch umgesetzt. Der Schrittmotor wird mithilfe eines Treibers angesteuert und kann über die Bedienelemente in verschiedenen Geschwindigkeitsstufen betrieben werden. Des Weiteren ist ein Geschwindigkeitssensor Typ LM393 verbaut, mit dem die tatsächliche Geschwindigkeit des Schrittmotors gemessen werden kann.</t>
+  </si>
+  <si>
+    <t>LINK GITHUB HIER EINFÜGEN</t>
+  </si>
+  <si>
+    <t>Hannah</t>
+  </si>
+  <si>
+    <t>Mey</t>
+  </si>
+  <si>
+    <t>Matrikelnummer</t>
+  </si>
+  <si>
+    <t>hannah-m12</t>
+  </si>
+  <si>
+    <t>hannah.mey@stud.hs-emden-leer.de</t>
+  </si>
+  <si>
+    <t>hannah.mey123@gmail.com</t>
+  </si>
+  <si>
+    <t>Maschinenbau und Design</t>
+  </si>
+  <si>
+    <t>Automation</t>
+  </si>
+  <si>
+    <t>12.03.2000</t>
+  </si>
+  <si>
+    <t>Jessica</t>
+  </si>
+  <si>
+    <t>Perewersenko</t>
+  </si>
+  <si>
+    <t>jessica.perewersenko@stud.hs-emden-leer.de</t>
+  </si>
+  <si>
+    <t>Chantal</t>
+  </si>
+  <si>
+    <t>Crety</t>
+  </si>
+  <si>
+    <r>
+      <t>7024</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>xxx</t>
+    </r>
+  </si>
+  <si>
+    <t>kthxjessy</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>&lt;Hochschule Emden/Leer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Fachbereich Technik&gt;</t>
+  </si>
+  <si>
+    <t>xxxx</t>
+  </si>
+  <si>
+    <t>xxxxxx</t>
+  </si>
+  <si>
+    <t>chantal.crety@stud.hs-emden-leer.de</t>
+  </si>
+  <si>
+    <t>chanti-logic</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="10" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -303,6 +335,25 @@
       <color theme="10"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -358,8 +409,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+  <cellXfs count="30">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -372,41 +423,47 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -1537,7 +1594,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B3:D16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="12.95" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1546,11 +1603,11 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:4" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
     </row>
     <row r="7" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
@@ -1581,7 +1638,7 @@
     </row>
     <row r="11" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
@@ -1592,12 +1649,12 @@
         <v>5</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
@@ -1608,12 +1665,12 @@
         <v>5</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
@@ -1624,7 +1681,7 @@
         <v>5</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1632,31 +1689,33 @@
     <mergeCell ref="B3:D3"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="D10" location="'Project'!R1C1" display="Project"/>
-    <hyperlink ref="D12" location="'Student 1'!R1C1" display="Student 1"/>
-    <hyperlink ref="D14" location="'Student 2'!R1C1" display="Student 2"/>
-    <hyperlink ref="D16" location="'Student 3'!R1C1" display="Student 3"/>
+    <hyperlink ref="D10" location="'Project'!R1C1" display="Project" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="D12" location="'Student 1'!R1C1" display="Student 1" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="D14" location="'Student 2'!R1C1" display="Student 2" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="D16" location="'Student 3'!R1C1" display="Student 3" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.85546875" style="5" customWidth="1"/>
-    <col min="2" max="6" width="11.42578125" style="5" customWidth="1"/>
+    <col min="1" max="1" width="37.42578125" style="5" customWidth="1"/>
+    <col min="2" max="2" width="31" style="5" customWidth="1"/>
+    <col min="3" max="3" width="66" style="5" customWidth="1"/>
+    <col min="4" max="6" width="11.42578125" style="5" customWidth="1"/>
     <col min="7" max="16384" width="11.42578125" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="61.9" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="21" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
+      <c r="A1" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
     </row>
@@ -1676,7 +1735,7 @@
     </row>
     <row r="4" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -1684,17 +1743,17 @@
       <c r="E4" s="6"/>
     </row>
     <row r="5" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="23" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="24"/>
-      <c r="C5" s="24"/>
+      <c r="A5" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -1702,8 +1761,8 @@
       <c r="E6" s="6"/>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="25" t="s">
-        <v>67</v>
+      <c r="A7" s="29" t="s">
+        <v>52</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -1737,7 +1796,7 @@
     <mergeCell ref="A5:C5"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A7" r:id="rId1"/>
+    <hyperlink ref="A7" r:id="rId1" display="ML24-04 Keyword Spotting with an Arduino Nano 33 BLE Sense" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740200000000005" bottom="0.78740200000000005" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -1748,17 +1807,17 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="47.28515625" style="9" customWidth="1"/>
-    <col min="2" max="2" width="46.85546875" style="9" customWidth="1"/>
-    <col min="3" max="3" width="33.140625" style="9" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" style="9" customWidth="1"/>
-    <col min="5" max="5" width="43.85546875" style="9" customWidth="1"/>
-    <col min="6" max="7" width="8.85546875" style="9" customWidth="1"/>
-    <col min="8" max="16384" width="8.85546875" style="9"/>
+    <col min="1" max="1" width="47.28515625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="46.85546875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="33.140625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="16.140625" style="5" customWidth="1"/>
+    <col min="5" max="5" width="43.85546875" style="5" customWidth="1"/>
+    <col min="6" max="7" width="8.85546875" style="5" customWidth="1"/>
+    <col min="8" max="16384" width="8.85546875" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1778,8 +1837,8 @@
       <c r="F2" s="6"/>
     </row>
     <row r="3" spans="1:6" ht="28.9" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="10" t="s">
-        <v>11</v>
+      <c r="A3" s="9" t="s">
+        <v>9</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -1789,36 +1848,48 @@
     </row>
     <row r="4" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="E4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="F4" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>17</v>
-      </c>
     </row>
     <row r="5" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="6"/>
+      <c r="A5" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" s="10">
+        <v>7024688</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="F5" s="23" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="6" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6"/>
       <c r="B6" s="6"/>
-      <c r="C6" s="12"/>
+      <c r="C6" s="11"/>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
@@ -1833,10 +1904,10 @@
     </row>
     <row r="8" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>19</v>
+        <v>59</v>
       </c>
       <c r="C8" s="6"/>
       <c r="D8" s="6"/>
@@ -1853,9 +1924,11 @@
     </row>
     <row r="10" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="13"/>
+        <v>17</v>
+      </c>
+      <c r="B10" s="12">
+        <v>4</v>
+      </c>
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
       <c r="E10" s="6"/>
@@ -1871,9 +1944,11 @@
     </row>
     <row r="12" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="14"/>
+        <v>18</v>
+      </c>
+      <c r="B12" s="13">
+        <v>45735</v>
+      </c>
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
@@ -1881,9 +1956,11 @@
     </row>
     <row r="13" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="14"/>
+        <v>19</v>
+      </c>
+      <c r="B13" s="13">
+        <v>45849</v>
+      </c>
       <c r="C13" s="6"/>
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
@@ -1899,9 +1976,11 @@
     </row>
     <row r="15" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B15" s="6"/>
+        <v>20</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>60</v>
+      </c>
       <c r="C15" s="6"/>
       <c r="D15" s="6"/>
       <c r="E15" s="6"/>
@@ -1909,10 +1988,10 @@
     </row>
     <row r="16" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B16" s="13">
-        <v>10</v>
+        <v>21</v>
+      </c>
+      <c r="B16" s="12">
+        <v>2</v>
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="6"/>
@@ -1937,9 +2016,11 @@
     </row>
     <row r="19" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B19" s="8"/>
+        <v>22</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>61</v>
+      </c>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
@@ -1954,8 +2035,8 @@
       <c r="F20" s="6"/>
     </row>
     <row r="21" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="15" t="s">
-        <v>26</v>
+      <c r="A21" s="14" t="s">
+        <v>23</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -1965,7 +2046,7 @@
     </row>
     <row r="22" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="6"/>
@@ -1975,7 +2056,7 @@
     </row>
     <row r="23" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="6"/>
@@ -1993,10 +2074,10 @@
     </row>
     <row r="25" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
@@ -2006,7 +2087,7 @@
     <row r="26" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6"/>
       <c r="B26" s="8" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
@@ -2016,7 +2097,7 @@
     <row r="27" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6"/>
       <c r="B27" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
@@ -2025,10 +2106,10 @@
     </row>
     <row r="28" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
@@ -2037,10 +2118,10 @@
     </row>
     <row r="29" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
@@ -2065,7 +2146,7 @@
     </row>
     <row r="32" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B32" s="6"/>
       <c r="C32" s="6"/>
@@ -2075,7 +2156,7 @@
     </row>
     <row r="33" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B33" s="8"/>
       <c r="C33" s="6"/>
@@ -2085,7 +2166,7 @@
     </row>
     <row r="34" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B34" s="8"/>
       <c r="C34" s="6"/>
@@ -2095,7 +2176,7 @@
     </row>
     <row r="35" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="6"/>
@@ -2104,7 +2185,7 @@
       <c r="F35" s="6"/>
     </row>
     <row r="36" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="16"/>
+      <c r="A36" s="15"/>
       <c r="B36" s="6"/>
       <c r="C36" s="6"/>
       <c r="D36" s="6"/>
@@ -2112,8 +2193,8 @@
       <c r="F36" s="6"/>
     </row>
     <row r="37" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="15" t="s">
-        <v>44</v>
+      <c r="A37" s="14" t="s">
+        <v>38</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -2123,10 +2204,10 @@
     </row>
     <row r="38" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="7" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C38" s="6"/>
       <c r="D38" s="6"/>
@@ -2135,10 +2216,10 @@
     </row>
     <row r="39" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C39" s="6"/>
       <c r="D39" s="6"/>
@@ -2147,10 +2228,10 @@
     </row>
     <row r="40" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="7" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="6"/>
@@ -2158,7 +2239,7 @@
       <c r="F40" s="6"/>
     </row>
     <row r="41" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="16"/>
+      <c r="A41" s="15"/>
       <c r="B41" s="6"/>
       <c r="C41" s="6"/>
       <c r="D41" s="6"/>
@@ -2166,7 +2247,7 @@
       <c r="F41" s="6"/>
     </row>
     <row r="42" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="16"/>
+      <c r="A42" s="15"/>
       <c r="B42" s="6"/>
       <c r="C42" s="6"/>
       <c r="D42" s="6"/>
@@ -2174,7 +2255,7 @@
       <c r="F42" s="6"/>
     </row>
     <row r="43" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="16"/>
+      <c r="A43" s="15"/>
       <c r="B43" s="6"/>
       <c r="C43" s="6"/>
       <c r="D43" s="6"/>
@@ -2182,8 +2263,8 @@
       <c r="F43" s="6"/>
     </row>
     <row r="44" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="15" t="s">
-        <v>50</v>
+      <c r="A44" s="14" t="s">
+        <v>44</v>
       </c>
       <c r="B44" s="6"/>
       <c r="C44" s="6"/>
@@ -2193,11 +2274,9 @@
     </row>
     <row r="45" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="B45" s="8" t="s">
-        <v>51</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="B45" s="8"/>
       <c r="C45" s="6"/>
       <c r="D45" s="6"/>
       <c r="E45" s="6"/>
@@ -2205,11 +2284,9 @@
     </row>
     <row r="46" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B46" s="8" t="s">
-        <v>52</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="B46" s="8"/>
       <c r="C46" s="6"/>
       <c r="D46" s="6"/>
       <c r="E46" s="6"/>
@@ -2217,18 +2294,16 @@
     </row>
     <row r="47" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B47" s="8" t="s">
-        <v>53</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="B47" s="8"/>
       <c r="C47" s="6"/>
       <c r="D47" s="6"/>
       <c r="E47" s="6"/>
       <c r="F47" s="6"/>
     </row>
     <row r="48" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="16"/>
+      <c r="A48" s="15"/>
       <c r="B48" s="6"/>
       <c r="C48" s="6"/>
       <c r="D48" s="6"/>
@@ -2236,7 +2311,7 @@
       <c r="F48" s="6"/>
     </row>
     <row r="49" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="16"/>
+      <c r="A49" s="15"/>
       <c r="B49" s="6"/>
       <c r="C49" s="6"/>
       <c r="D49" s="6"/>
@@ -2245,10 +2320,10 @@
     </row>
     <row r="50" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="C50" s="6"/>
       <c r="D50" s="6"/>
@@ -2257,12 +2332,14 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"Technical Management,Business Intelligen ans Data Analytics,Maschinenbau,Indin,IBS,Maschinenbau und Design,Maschinenbau und Design im Praxisverbund,Engineering Physics,other"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="B40" r:id="rId1"/>
+    <hyperlink ref="B40" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
+    <hyperlink ref="E5" r:id="rId2" xr:uid="{E2F13D68-51B4-40B7-96C1-008B965F21C7}"/>
+    <hyperlink ref="F5" r:id="rId3" xr:uid="{59CFE6B4-EAA6-4D0F-9362-2D5843AC9AFE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -2273,18 +2350,18 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.42578125" style="17" customWidth="1"/>
-    <col min="2" max="2" width="46.85546875" style="17" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" style="17" customWidth="1"/>
-    <col min="4" max="4" width="15.42578125" style="17" customWidth="1"/>
-    <col min="5" max="5" width="44.42578125" style="17" customWidth="1"/>
-    <col min="6" max="6" width="21.85546875" style="17" customWidth="1"/>
-    <col min="7" max="7" width="11.42578125" style="17" customWidth="1"/>
-    <col min="8" max="16384" width="11.42578125" style="17"/>
+    <col min="1" max="1" width="29.42578125" style="5" customWidth="1"/>
+    <col min="2" max="2" width="46.85546875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="14.85546875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="15.42578125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="44.42578125" style="5" customWidth="1"/>
+    <col min="6" max="6" width="21.85546875" style="5" customWidth="1"/>
+    <col min="7" max="7" width="11.42578125" style="5" customWidth="1"/>
+    <col min="8" max="16384" width="11.42578125" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2304,8 +2381,8 @@
       <c r="F2" s="6"/>
     </row>
     <row r="3" spans="1:6" ht="28.9" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="10" t="s">
-        <v>11</v>
+      <c r="A3" s="9" t="s">
+        <v>9</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -2315,36 +2392,48 @@
     </row>
     <row r="4" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="E4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="F4" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>17</v>
-      </c>
     </row>
     <row r="5" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
+      <c r="A5" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="F5" s="26" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="6" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6"/>
       <c r="B6" s="6"/>
-      <c r="C6" s="12"/>
+      <c r="C6" s="11"/>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
@@ -2359,10 +2448,10 @@
     </row>
     <row r="8" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>19</v>
+        <v>59</v>
       </c>
       <c r="C8" s="6"/>
       <c r="D8" s="6"/>
@@ -2379,10 +2468,10 @@
     </row>
     <row r="10" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="13">
-        <v>1</v>
+        <v>17</v>
+      </c>
+      <c r="B10" s="12">
+        <v>4</v>
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
@@ -2399,9 +2488,11 @@
     </row>
     <row r="12" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="14"/>
+        <v>18</v>
+      </c>
+      <c r="B12" s="13">
+        <v>45735</v>
+      </c>
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
@@ -2409,9 +2500,11 @@
     </row>
     <row r="13" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="14"/>
+        <v>19</v>
+      </c>
+      <c r="B13" s="13">
+        <v>45849</v>
+      </c>
       <c r="C13" s="6"/>
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
@@ -2427,10 +2520,10 @@
     </row>
     <row r="15" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>57</v>
+        <v>20</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>60</v>
       </c>
       <c r="C15" s="6"/>
       <c r="D15" s="6"/>
@@ -2439,10 +2532,10 @@
     </row>
     <row r="16" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B16" s="13">
-        <v>10</v>
+        <v>21</v>
+      </c>
+      <c r="B16" s="12">
+        <v>2</v>
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="6"/>
@@ -2467,9 +2560,11 @@
     </row>
     <row r="19" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B19" s="8"/>
+        <v>22</v>
+      </c>
+      <c r="B19" s="26" t="s">
+        <v>72</v>
+      </c>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
@@ -2484,8 +2579,8 @@
       <c r="F20" s="6"/>
     </row>
     <row r="21" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="15" t="s">
-        <v>26</v>
+      <c r="A21" s="14" t="s">
+        <v>23</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -2495,7 +2590,7 @@
     </row>
     <row r="22" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="6"/>
@@ -2505,7 +2600,7 @@
     </row>
     <row r="23" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="6"/>
@@ -2523,10 +2618,10 @@
     </row>
     <row r="25" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>58</v>
+        <v>26</v>
+      </c>
+      <c r="B25" s="25" t="s">
+        <v>70</v>
       </c>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
@@ -2535,8 +2630,8 @@
     </row>
     <row r="26" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6"/>
-      <c r="B26" s="8" t="s">
-        <v>59</v>
+      <c r="B26" s="25" t="s">
+        <v>71</v>
       </c>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
@@ -2546,7 +2641,7 @@
     <row r="27" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6"/>
       <c r="B27" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
@@ -2555,10 +2650,10 @@
     </row>
     <row r="28" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
@@ -2567,10 +2662,10 @@
     </row>
     <row r="29" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
@@ -2595,7 +2690,7 @@
     </row>
     <row r="32" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B32" s="6"/>
       <c r="C32" s="6"/>
@@ -2605,7 +2700,7 @@
     </row>
     <row r="33" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B33" s="8"/>
       <c r="C33" s="6"/>
@@ -2615,7 +2710,7 @@
     </row>
     <row r="34" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B34" s="8"/>
       <c r="C34" s="6"/>
@@ -2625,7 +2720,7 @@
     </row>
     <row r="35" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="6"/>
@@ -2634,7 +2729,7 @@
       <c r="F35" s="6"/>
     </row>
     <row r="36" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="16"/>
+      <c r="A36" s="15"/>
       <c r="B36" s="6"/>
       <c r="C36" s="6"/>
       <c r="D36" s="6"/>
@@ -2642,8 +2737,8 @@
       <c r="F36" s="6"/>
     </row>
     <row r="37" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="15" t="s">
-        <v>44</v>
+      <c r="A37" s="14" t="s">
+        <v>38</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -2653,10 +2748,10 @@
     </row>
     <row r="38" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="7" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C38" s="6"/>
       <c r="D38" s="6"/>
@@ -2665,10 +2760,10 @@
     </row>
     <row r="39" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C39" s="6"/>
       <c r="D39" s="6"/>
@@ -2677,10 +2772,10 @@
     </row>
     <row r="40" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="7" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="6"/>
@@ -2688,7 +2783,7 @@
       <c r="F40" s="6"/>
     </row>
     <row r="41" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="16"/>
+      <c r="A41" s="15"/>
       <c r="B41" s="6"/>
       <c r="C41" s="6"/>
       <c r="D41" s="6"/>
@@ -2696,7 +2791,7 @@
       <c r="F41" s="6"/>
     </row>
     <row r="42" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="16"/>
+      <c r="A42" s="15"/>
       <c r="B42" s="6"/>
       <c r="C42" s="6"/>
       <c r="D42" s="6"/>
@@ -2704,7 +2799,7 @@
       <c r="F42" s="6"/>
     </row>
     <row r="43" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="16"/>
+      <c r="A43" s="15"/>
       <c r="B43" s="6"/>
       <c r="C43" s="6"/>
       <c r="D43" s="6"/>
@@ -2712,8 +2807,8 @@
       <c r="F43" s="6"/>
     </row>
     <row r="44" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="15" t="s">
-        <v>50</v>
+      <c r="A44" s="14" t="s">
+        <v>44</v>
       </c>
       <c r="B44" s="6"/>
       <c r="C44" s="6"/>
@@ -2723,11 +2818,9 @@
     </row>
     <row r="45" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="B45" s="8" t="s">
-        <v>51</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="B45" s="8"/>
       <c r="C45" s="6"/>
       <c r="D45" s="6"/>
       <c r="E45" s="6"/>
@@ -2735,11 +2828,9 @@
     </row>
     <row r="46" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B46" s="8" t="s">
-        <v>52</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="B46" s="8"/>
       <c r="C46" s="6"/>
       <c r="D46" s="6"/>
       <c r="E46" s="6"/>
@@ -2747,18 +2838,16 @@
     </row>
     <row r="47" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B47" s="8" t="s">
-        <v>53</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="B47" s="8"/>
       <c r="C47" s="6"/>
       <c r="D47" s="6"/>
       <c r="E47" s="6"/>
       <c r="F47" s="6"/>
     </row>
     <row r="48" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="16"/>
+      <c r="A48" s="15"/>
       <c r="B48" s="6"/>
       <c r="C48" s="6"/>
       <c r="D48" s="6"/>
@@ -2766,7 +2855,7 @@
       <c r="F48" s="6"/>
     </row>
     <row r="49" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="16"/>
+      <c r="A49" s="15"/>
       <c r="B49" s="6"/>
       <c r="C49" s="6"/>
       <c r="D49" s="6"/>
@@ -2775,10 +2864,10 @@
     </row>
     <row r="50" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="C50" s="6"/>
       <c r="D50" s="6"/>
@@ -2787,12 +2876,13 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"Technical Management,Business Intelligen ans Data Analytics,Maschinenbau,Indin,IBS,Maschinenbau und Design,Maschinenbau und Design im Praxisverbund,Engineering Physics,other"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="B40" r:id="rId1"/>
+    <hyperlink ref="B40" r:id="rId1" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
+    <hyperlink ref="E5" r:id="rId2" xr:uid="{003C16DA-B661-456F-9CD6-082A96752A15}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740200000000005" bottom="0.78740200000000005" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -2803,16 +2893,17 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.140625" style="18" customWidth="1"/>
-    <col min="2" max="2" width="49.7109375" style="18" customWidth="1"/>
-    <col min="3" max="3" width="15.42578125" style="18" customWidth="1"/>
-    <col min="4" max="5" width="16.140625" style="18" customWidth="1"/>
-    <col min="6" max="7" width="11.42578125" style="18" customWidth="1"/>
-    <col min="8" max="16384" width="11.42578125" style="18"/>
+    <col min="1" max="1" width="29.140625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="49.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" style="5" customWidth="1"/>
+    <col min="4" max="4" width="16.140625" style="5" customWidth="1"/>
+    <col min="5" max="5" width="39.28515625" style="5" customWidth="1"/>
+    <col min="6" max="7" width="11.42578125" style="5" customWidth="1"/>
+    <col min="8" max="16384" width="11.42578125" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2832,8 +2923,8 @@
       <c r="F2" s="6"/>
     </row>
     <row r="3" spans="1:6" ht="28.9" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="10" t="s">
-        <v>11</v>
+      <c r="A3" s="9" t="s">
+        <v>9</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -2843,42 +2934,48 @@
     </row>
     <row r="4" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="E4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="F4" s="7" t="s">
         <v>15</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="C5" s="11">
-        <v>1234567</v>
-      </c>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
+        <v>66</v>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="27" t="s">
+        <v>75</v>
+      </c>
+      <c r="E5" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="F5" s="28" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="6" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6"/>
       <c r="B6" s="6"/>
-      <c r="C6" s="12"/>
+      <c r="C6" s="11"/>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
@@ -2893,9 +2990,11 @@
     </row>
     <row r="8" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="6"/>
+        <v>16</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>59</v>
+      </c>
       <c r="C8" s="6"/>
       <c r="D8" s="6"/>
       <c r="E8" s="6"/>
@@ -2911,10 +3010,10 @@
     </row>
     <row r="10" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="13">
-        <v>7</v>
+        <v>17</v>
+      </c>
+      <c r="B10" s="12">
+        <v>4</v>
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
@@ -2931,10 +3030,10 @@
     </row>
     <row r="12" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="14">
-        <v>45351</v>
+        <v>18</v>
+      </c>
+      <c r="B12" s="13">
+        <v>45735</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
@@ -2943,10 +3042,10 @@
     </row>
     <row r="13" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="14">
-        <v>45594</v>
+        <v>19</v>
+      </c>
+      <c r="B13" s="13">
+        <v>45849</v>
       </c>
       <c r="C13" s="6"/>
       <c r="D13" s="6"/>
@@ -2963,9 +3062,11 @@
     </row>
     <row r="15" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B15" s="6"/>
+        <v>20</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>60</v>
+      </c>
       <c r="C15" s="6"/>
       <c r="D15" s="6"/>
       <c r="E15" s="6"/>
@@ -2973,10 +3074,10 @@
     </row>
     <row r="16" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>63</v>
+        <v>21</v>
+      </c>
+      <c r="B16" s="25" t="s">
+        <v>69</v>
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="6"/>
@@ -3001,10 +3102,10 @@
     </row>
     <row r="19" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>64</v>
+        <v>22</v>
+      </c>
+      <c r="B19" s="26" t="s">
+        <v>49</v>
       </c>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
@@ -3020,8 +3121,8 @@
       <c r="F20" s="6"/>
     </row>
     <row r="21" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="15" t="s">
-        <v>26</v>
+      <c r="A21" s="14" t="s">
+        <v>23</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -3031,11 +3132,9 @@
     </row>
     <row r="22" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>65</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="B22" s="8"/>
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
@@ -3043,11 +3142,9 @@
     </row>
     <row r="23" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>36</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="B23" s="8"/>
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
@@ -3063,10 +3160,10 @@
     </row>
     <row r="25" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>58</v>
+        <v>26</v>
+      </c>
+      <c r="B25" s="25" t="s">
+        <v>70</v>
       </c>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
@@ -3075,8 +3172,8 @@
     </row>
     <row r="26" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6"/>
-      <c r="B26" s="8" t="s">
-        <v>59</v>
+      <c r="B26" s="25" t="s">
+        <v>71</v>
       </c>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
@@ -3086,7 +3183,7 @@
     <row r="27" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6"/>
       <c r="B27" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
@@ -3095,10 +3192,10 @@
     </row>
     <row r="28" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
@@ -3107,10 +3204,10 @@
     </row>
     <row r="29" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
@@ -3135,7 +3232,7 @@
     </row>
     <row r="32" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B32" s="6"/>
       <c r="C32" s="6"/>
@@ -3145,11 +3242,9 @@
     </row>
     <row r="33" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>39</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="B33" s="8"/>
       <c r="C33" s="6"/>
       <c r="D33" s="6"/>
       <c r="E33" s="6"/>
@@ -3157,11 +3252,9 @@
     </row>
     <row r="34" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B34" s="8" t="s">
-        <v>41</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="B34" s="8"/>
       <c r="C34" s="6"/>
       <c r="D34" s="6"/>
       <c r="E34" s="6"/>
@@ -3169,18 +3262,16 @@
     </row>
     <row r="35" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="B35" s="8" t="s">
-        <v>43</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="B35" s="8"/>
       <c r="C35" s="6"/>
       <c r="D35" s="6"/>
       <c r="E35" s="6"/>
       <c r="F35" s="6"/>
     </row>
     <row r="36" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="16"/>
+      <c r="A36" s="15"/>
       <c r="B36" s="6"/>
       <c r="C36" s="6"/>
       <c r="D36" s="6"/>
@@ -3188,8 +3279,8 @@
       <c r="F36" s="6"/>
     </row>
     <row r="37" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="15" t="s">
-        <v>44</v>
+      <c r="A37" s="14" t="s">
+        <v>38</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -3199,10 +3290,10 @@
     </row>
     <row r="38" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="7" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>66</v>
+        <v>40</v>
       </c>
       <c r="C38" s="6"/>
       <c r="D38" s="6"/>
@@ -3211,10 +3302,10 @@
     </row>
     <row r="39" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="C39" s="6"/>
       <c r="D39" s="6"/>
@@ -3223,10 +3314,10 @@
     </row>
     <row r="40" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="7" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="6"/>
@@ -3234,7 +3325,7 @@
       <c r="F40" s="6"/>
     </row>
     <row r="41" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="16"/>
+      <c r="A41" s="15"/>
       <c r="B41" s="6"/>
       <c r="C41" s="6"/>
       <c r="D41" s="6"/>
@@ -3242,7 +3333,7 @@
       <c r="F41" s="6"/>
     </row>
     <row r="42" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="16"/>
+      <c r="A42" s="15"/>
       <c r="B42" s="6"/>
       <c r="C42" s="6"/>
       <c r="D42" s="6"/>
@@ -3250,7 +3341,7 @@
       <c r="F42" s="6"/>
     </row>
     <row r="43" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="16"/>
+      <c r="A43" s="15"/>
       <c r="B43" s="6"/>
       <c r="C43" s="6"/>
       <c r="D43" s="6"/>
@@ -3258,8 +3349,8 @@
       <c r="F43" s="6"/>
     </row>
     <row r="44" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="15" t="s">
-        <v>50</v>
+      <c r="A44" s="14" t="s">
+        <v>44</v>
       </c>
       <c r="B44" s="6"/>
       <c r="C44" s="6"/>
@@ -3269,11 +3360,9 @@
     </row>
     <row r="45" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="B45" s="8" t="s">
-        <v>51</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="B45" s="8"/>
       <c r="C45" s="6"/>
       <c r="D45" s="6"/>
       <c r="E45" s="6"/>
@@ -3281,11 +3370,9 @@
     </row>
     <row r="46" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B46" s="8" t="s">
-        <v>52</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="B46" s="8"/>
       <c r="C46" s="6"/>
       <c r="D46" s="6"/>
       <c r="E46" s="6"/>
@@ -3293,18 +3380,16 @@
     </row>
     <row r="47" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B47" s="8" t="s">
-        <v>53</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="B47" s="8"/>
       <c r="C47" s="6"/>
       <c r="D47" s="6"/>
       <c r="E47" s="6"/>
       <c r="F47" s="6"/>
     </row>
     <row r="48" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="16"/>
+      <c r="A48" s="15"/>
       <c r="B48" s="6"/>
       <c r="C48" s="6"/>
       <c r="D48" s="6"/>
@@ -3312,7 +3397,7 @@
       <c r="F48" s="6"/>
     </row>
     <row r="49" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="16"/>
+      <c r="A49" s="15"/>
       <c r="B49" s="6"/>
       <c r="C49" s="6"/>
       <c r="D49" s="6"/>
@@ -3321,10 +3406,10 @@
     </row>
     <row r="50" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="C50" s="6"/>
       <c r="D50" s="6"/>
@@ -3333,12 +3418,16 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8" xr:uid="{00000000-0002-0000-0400-000000000000}">
       <formula1>"Technical Management,Business Intelligen ans Data Analytics,Maschinenbau,Indin,IBS,Maschinenbau und Design,Maschinenbau und Design im Praxisverbund,Engineering Physics,other"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="B40" r:id="rId1" xr:uid="{D3CE74DB-3372-4D8E-8038-3ACB444024CD}"/>
+    <hyperlink ref="E5" r:id="rId2" xr:uid="{D4630012-1892-431F-AA1D-FF1C1B9B5231}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740200000000005" bottom="0.78740200000000005" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>

</xml_diff>